<commit_message>
Update database configuration, add new routes for previewing financial statements, and enhance financial statement and general ledger views. Include new Excel files for financial statements and trial balance.
</commit_message>
<xml_diff>
--- a/assets/templates/fpc.xlsx
+++ b/assets/templates/fpc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\jev-jaro\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CF5565-6470-4F06-B61F-4A2ACA01D452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A32D1D1-769F-4BB5-A0E1-989D2DD2365E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{3D37FFD8-D4A5-48D1-ADF7-7A80C174BD04}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{3D37FFD8-D4A5-48D1-ADF7-7A80C174BD04}"/>
   </bookViews>
   <sheets>
     <sheet name="Detailed Financial Performance" sheetId="2" r:id="rId1"/>
@@ -3713,11 +3713,11 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3725,8 +3725,8 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3734,29 +3734,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3776,53 +3758,41 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3848,16 +3818,46 @@
     <xf numFmtId="0" fontId="41" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4544,9 +4544,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4584,7 +4584,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4690,7 +4690,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4832,7 +4832,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -10026,45 +10026,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="158" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="158"/>
-      <c r="C1" s="158"/>
-      <c r="D1" s="158"/>
-      <c r="E1" s="158"/>
-      <c r="F1" s="158"/>
+      <c r="A1" s="162" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="158" t="s">
+      <c r="A2" s="162" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="158"/>
-      <c r="C2" s="158"/>
-      <c r="D2" s="158"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="158"/>
+      <c r="B2" s="162"/>
+      <c r="C2" s="162"/>
+      <c r="D2" s="162"/>
+      <c r="E2" s="162"/>
+      <c r="F2" s="162"/>
     </row>
     <row r="3" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="159" t="s">
+      <c r="A3" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="159"/>
-      <c r="C3" s="159"/>
-      <c r="D3" s="159"/>
-      <c r="E3" s="159"/>
-      <c r="F3" s="159"/>
+      <c r="B3" s="165"/>
+      <c r="C3" s="165"/>
+      <c r="D3" s="165"/>
+      <c r="E3" s="165"/>
+      <c r="F3" s="165"/>
     </row>
     <row r="4" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="158">
+      <c r="A4" s="162">
         <f>'Detailed Financial Performance'!A9</f>
         <v>0</v>
       </c>
-      <c r="B4" s="158"/>
-      <c r="C4" s="158"/>
-      <c r="D4" s="158"/>
-      <c r="E4" s="158"/>
-      <c r="F4" s="158"/>
+      <c r="B4" s="162"/>
+      <c r="C4" s="162"/>
+      <c r="D4" s="162"/>
+      <c r="E4" s="162"/>
+      <c r="F4" s="162"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="163" t="s">
@@ -10087,15 +10087,15 @@
       <c r="F6" s="164"/>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="159">
+      <c r="A7" s="165">
         <f>'Detailed Financial Performance'!A12</f>
         <v>0</v>
       </c>
-      <c r="B7" s="159"/>
-      <c r="C7" s="159"/>
-      <c r="D7" s="159"/>
-      <c r="E7" s="159"/>
-      <c r="F7" s="159"/>
+      <c r="B7" s="165"/>
+      <c r="C7" s="165"/>
+      <c r="D7" s="165"/>
+      <c r="E7" s="165"/>
+      <c r="F7" s="165"/>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
@@ -10105,11 +10105,11 @@
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="159" t="s">
+      <c r="A9" s="165" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="158"/>
-      <c r="C9" s="158"/>
+      <c r="B9" s="162"/>
+      <c r="C9" s="162"/>
       <c r="D9" s="2">
         <f>'Detailed Financial Performance'!F13</f>
         <v>0</v>
@@ -10140,11 +10140,11 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="165" t="s">
+      <c r="A10" s="166" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="165"/>
-      <c r="C10" s="165"/>
+      <c r="B10" s="166"/>
+      <c r="C10" s="166"/>
       <c r="D10" s="5"/>
       <c r="E10" s="1"/>
     </row>
@@ -10479,7 +10479,7 @@
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="44">
-        <f>'Detailed Financial Performance'!F234</f>
+        <f>'Detailed Financial Performance'!F234+'Detailed Financial Performance'!F300+'Detailed Financial Performance'!F304</f>
         <v>0</v>
       </c>
       <c r="E21" s="44">
@@ -10613,11 +10613,11 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="21" x14ac:dyDescent="0.25">
-      <c r="A25" s="162" t="s">
+      <c r="A25" s="158" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="162"/>
-      <c r="C25" s="162"/>
+      <c r="B25" s="158"/>
+      <c r="C25" s="158"/>
       <c r="D25" s="47">
         <f>D18-D24</f>
         <v>0</v>
@@ -10649,10 +10649,10 @@
     </row>
     <row r="26" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
-      <c r="B26" s="162" t="s">
+      <c r="B26" s="158" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="162"/>
+      <c r="C26" s="158"/>
       <c r="D26" s="44"/>
       <c r="E26" s="1"/>
     </row>
@@ -10727,11 +10727,11 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="21" x14ac:dyDescent="0.25">
-      <c r="A29" s="166" t="s">
+      <c r="A29" s="159" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="166"/>
-      <c r="C29" s="166"/>
+      <c r="B29" s="159"/>
+      <c r="C29" s="159"/>
       <c r="D29" s="47">
         <f>D25+D28</f>
         <v>0</v>
@@ -10788,8 +10788,8 @@
     </row>
     <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
-      <c r="B33" s="162"/>
-      <c r="C33" s="162"/>
+      <c r="B33" s="158"/>
+      <c r="C33" s="158"/>
       <c r="D33" s="13" t="s">
         <v>28</v>
       </c>
@@ -10806,11 +10806,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A25:C25"/>
@@ -10819,11 +10819,11 @@
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="76" orientation="portrait" r:id="rId1"/>
@@ -20531,46 +20531,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="158" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="158"/>
-      <c r="C1" s="158"/>
-      <c r="D1" s="158"/>
-      <c r="E1" s="158"/>
-      <c r="F1" s="158"/>
-      <c r="G1" s="158"/>
+      <c r="A1" s="162" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
     </row>
     <row r="2" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="158" t="s">
+      <c r="A2" s="162" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="158"/>
-      <c r="C2" s="158"/>
-      <c r="D2" s="158"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="158"/>
-      <c r="G2" s="158"/>
+      <c r="B2" s="162"/>
+      <c r="C2" s="162"/>
+      <c r="D2" s="162"/>
+      <c r="E2" s="162"/>
+      <c r="F2" s="162"/>
+      <c r="G2" s="162"/>
     </row>
     <row r="3" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="159" t="s">
+      <c r="A3" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="159"/>
-      <c r="C3" s="159"/>
-      <c r="D3" s="159"/>
-      <c r="E3" s="159"/>
-      <c r="F3" s="159"/>
-      <c r="G3" s="159"/>
+      <c r="B3" s="165"/>
+      <c r="C3" s="165"/>
+      <c r="D3" s="165"/>
+      <c r="E3" s="165"/>
+      <c r="F3" s="165"/>
+      <c r="G3" s="165"/>
     </row>
     <row r="4" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="158"/>
-      <c r="B4" s="158"/>
-      <c r="C4" s="158"/>
-      <c r="D4" s="158"/>
-      <c r="E4" s="158"/>
-      <c r="F4" s="158"/>
-      <c r="G4" s="158"/>
+      <c r="A4" s="162"/>
+      <c r="B4" s="162"/>
+      <c r="C4" s="162"/>
+      <c r="D4" s="162"/>
+      <c r="E4" s="162"/>
+      <c r="F4" s="162"/>
+      <c r="G4" s="162"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="163" t="s">
@@ -20584,13 +20584,13 @@
       <c r="G5" s="163"/>
     </row>
     <row r="6" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="159"/>
-      <c r="B6" s="159"/>
-      <c r="C6" s="159"/>
-      <c r="D6" s="159"/>
-      <c r="E6" s="159"/>
-      <c r="F6" s="159"/>
-      <c r="G6" s="159"/>
+      <c r="A6" s="165"/>
+      <c r="B6" s="165"/>
+      <c r="C6" s="165"/>
+      <c r="D6" s="165"/>
+      <c r="E6" s="165"/>
+      <c r="F6" s="165"/>
+      <c r="G6" s="165"/>
     </row>
     <row r="7" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="164" t="s">
@@ -20604,20 +20604,20 @@
       <c r="G7" s="164"/>
     </row>
     <row r="8" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="168"/>
-      <c r="B8" s="168"/>
-      <c r="C8" s="168"/>
-      <c r="D8" s="168"/>
-      <c r="E8" s="168"/>
-      <c r="F8" s="168"/>
-      <c r="G8" s="168"/>
+      <c r="A8" s="177"/>
+      <c r="B8" s="177"/>
+      <c r="C8" s="177"/>
+      <c r="D8" s="177"/>
+      <c r="E8" s="177"/>
+      <c r="F8" s="177"/>
+      <c r="G8" s="177"/>
     </row>
     <row r="9" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="169" t="s">
+      <c r="A9" s="178" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="169"/>
-      <c r="C9" s="170"/>
+      <c r="B9" s="178"/>
+      <c r="C9" s="179"/>
       <c r="D9" s="82"/>
       <c r="E9" s="82"/>
       <c r="F9" s="82"/>
@@ -20626,12 +20626,12 @@
       <c r="I9" s="82"/>
     </row>
     <row r="10" spans="1:9" s="83" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="171" t="s">
+      <c r="A10" s="173" t="s">
         <v>343</v>
       </c>
-      <c r="B10" s="171"/>
-      <c r="C10" s="171"/>
-      <c r="D10" s="171"/>
+      <c r="B10" s="173"/>
+      <c r="C10" s="173"/>
+      <c r="D10" s="173"/>
       <c r="I10" s="84"/>
     </row>
     <row r="11" spans="1:9" s="83" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -20802,11 +20802,11 @@
       </c>
     </row>
     <row r="17" spans="1:9" s="83" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="172" t="s">
+      <c r="A17" s="174" t="s">
         <v>765</v>
       </c>
-      <c r="B17" s="172"/>
-      <c r="C17" s="172"/>
+      <c r="B17" s="174"/>
+      <c r="C17" s="174"/>
       <c r="D17" s="92">
         <f>SUM(D12:D16)</f>
         <v>0</v>
@@ -21041,11 +21041,11 @@
       <c r="I25" s="84"/>
     </row>
     <row r="26" spans="1:9" s="83" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="167" t="s">
+      <c r="A26" s="176" t="s">
         <v>769</v>
       </c>
-      <c r="B26" s="167"/>
-      <c r="C26" s="167"/>
+      <c r="B26" s="176"/>
+      <c r="C26" s="176"/>
       <c r="D26" s="97">
         <f>SUM(D19:D24)</f>
         <v>0</v>
@@ -21072,11 +21072,11 @@
       </c>
     </row>
     <row r="27" spans="1:9" s="83" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="176" t="s">
+      <c r="A27" s="170" t="s">
         <v>770</v>
       </c>
-      <c r="B27" s="177"/>
-      <c r="C27" s="178"/>
+      <c r="B27" s="171"/>
+      <c r="C27" s="172"/>
       <c r="D27" s="98">
         <f>D17+D26</f>
         <v>0</v>
@@ -21103,12 +21103,12 @@
       </c>
     </row>
     <row r="28" spans="1:9" s="83" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="171" t="s">
+      <c r="A28" s="173" t="s">
         <v>689</v>
       </c>
-      <c r="B28" s="171"/>
-      <c r="C28" s="171"/>
-      <c r="D28" s="171"/>
+      <c r="B28" s="173"/>
+      <c r="C28" s="173"/>
+      <c r="D28" s="173"/>
       <c r="E28" s="99"/>
       <c r="F28" s="99"/>
       <c r="G28" s="99"/>
@@ -21282,11 +21282,11 @@
       </c>
     </row>
     <row r="35" spans="1:9" s="83" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="172" t="s">
+      <c r="A35" s="174" t="s">
         <v>748</v>
       </c>
-      <c r="B35" s="172"/>
-      <c r="C35" s="172"/>
+      <c r="B35" s="174"/>
+      <c r="C35" s="174"/>
       <c r="D35" s="92">
         <f>SUM(D30:D34)</f>
         <v>0</v>
@@ -21449,11 +21449,11 @@
       </c>
     </row>
     <row r="41" spans="1:9" s="83" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="179" t="s">
+      <c r="A41" s="175" t="s">
         <v>774</v>
       </c>
-      <c r="B41" s="179"/>
-      <c r="C41" s="179"/>
+      <c r="B41" s="175"/>
+      <c r="C41" s="175"/>
       <c r="D41" s="101">
         <f>SUM(D37:D40)</f>
         <v>0</v>
@@ -21480,11 +21480,11 @@
       </c>
     </row>
     <row r="42" spans="1:9" s="83" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="176" t="s">
+      <c r="A42" s="170" t="s">
         <v>775</v>
       </c>
-      <c r="B42" s="177"/>
-      <c r="C42" s="178"/>
+      <c r="B42" s="171"/>
+      <c r="C42" s="172"/>
       <c r="D42" s="98">
         <f>SUM(D35+D41)</f>
         <v>0</v>
@@ -21511,12 +21511,12 @@
       </c>
     </row>
     <row r="43" spans="1:9" s="83" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="171" t="s">
+      <c r="A43" s="173" t="s">
         <v>753</v>
       </c>
-      <c r="B43" s="171"/>
-      <c r="C43" s="171"/>
-      <c r="D43" s="171"/>
+      <c r="B43" s="173"/>
+      <c r="C43" s="173"/>
+      <c r="D43" s="173"/>
       <c r="E43" s="99"/>
       <c r="F43" s="99"/>
       <c r="G43" s="99"/>
@@ -21585,11 +21585,11 @@
       </c>
     </row>
     <row r="46" spans="1:9" s="83" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="173" t="s">
+      <c r="A46" s="167" t="s">
         <v>777</v>
       </c>
-      <c r="B46" s="174"/>
-      <c r="C46" s="175"/>
+      <c r="B46" s="168"/>
+      <c r="C46" s="169"/>
       <c r="D46" s="102">
         <f>D42+D44</f>
         <v>0</v>
@@ -21652,8 +21652,8 @@
     </row>
     <row r="51" spans="1:9" s="106" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="5"/>
-      <c r="B51" s="162"/>
-      <c r="C51" s="162"/>
+      <c r="B51" s="158"/>
+      <c r="C51" s="158"/>
       <c r="E51" s="13" t="s">
         <v>28</v>
       </c>
@@ -21674,16 +21674,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A43:D43"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
@@ -21696,6 +21686,16 @@
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A43:D43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="51" orientation="portrait" r:id="rId1"/>
@@ -22353,101 +22353,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="204" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="204"/>
-      <c r="C1" s="204"/>
-      <c r="D1" s="204"/>
-      <c r="E1" s="204"/>
-      <c r="F1" s="204"/>
-      <c r="G1" s="204"/>
-      <c r="H1" s="204"/>
-      <c r="I1" s="204"/>
+      <c r="A1" s="181" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="181"/>
+      <c r="C1" s="181"/>
+      <c r="D1" s="181"/>
+      <c r="E1" s="181"/>
+      <c r="F1" s="181"/>
+      <c r="G1" s="181"/>
+      <c r="H1" s="181"/>
+      <c r="I1" s="181"/>
     </row>
     <row r="2" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="204" t="s">
+      <c r="A2" s="181" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="204"/>
-      <c r="C2" s="204"/>
-      <c r="D2" s="204"/>
-      <c r="E2" s="204"/>
-      <c r="F2" s="204"/>
-      <c r="G2" s="204"/>
-      <c r="H2" s="204"/>
-      <c r="I2" s="204"/>
+      <c r="B2" s="181"/>
+      <c r="C2" s="181"/>
+      <c r="D2" s="181"/>
+      <c r="E2" s="181"/>
+      <c r="F2" s="181"/>
+      <c r="G2" s="181"/>
+      <c r="H2" s="181"/>
+      <c r="I2" s="181"/>
     </row>
     <row r="3" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="205" t="s">
+      <c r="A3" s="182" t="s">
         <v>341</v>
       </c>
-      <c r="B3" s="205"/>
-      <c r="C3" s="205"/>
-      <c r="D3" s="205"/>
-      <c r="E3" s="205"/>
-      <c r="F3" s="205"/>
-      <c r="G3" s="205"/>
-      <c r="H3" s="205"/>
-      <c r="I3" s="205"/>
+      <c r="B3" s="182"/>
+      <c r="C3" s="182"/>
+      <c r="D3" s="182"/>
+      <c r="E3" s="182"/>
+      <c r="F3" s="182"/>
+      <c r="G3" s="182"/>
+      <c r="H3" s="182"/>
+      <c r="I3" s="182"/>
     </row>
     <row r="4" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="204"/>
-      <c r="B4" s="204"/>
-      <c r="C4" s="204"/>
-      <c r="D4" s="204"/>
-      <c r="E4" s="204"/>
-      <c r="F4" s="204"/>
-      <c r="G4" s="204"/>
-      <c r="H4" s="204"/>
-      <c r="I4" s="204"/>
+      <c r="A4" s="181"/>
+      <c r="B4" s="181"/>
+      <c r="C4" s="181"/>
+      <c r="D4" s="181"/>
+      <c r="E4" s="181"/>
+      <c r="F4" s="181"/>
+      <c r="G4" s="181"/>
+      <c r="H4" s="181"/>
+      <c r="I4" s="181"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="206" t="s">
+      <c r="A5" s="183" t="s">
         <v>778</v>
       </c>
-      <c r="B5" s="206"/>
-      <c r="C5" s="206"/>
-      <c r="D5" s="206"/>
-      <c r="E5" s="206"/>
-      <c r="F5" s="206"/>
-      <c r="G5" s="206"/>
-      <c r="H5" s="206"/>
-      <c r="I5" s="206"/>
+      <c r="B5" s="183"/>
+      <c r="C5" s="183"/>
+      <c r="D5" s="183"/>
+      <c r="E5" s="183"/>
+      <c r="F5" s="183"/>
+      <c r="G5" s="183"/>
+      <c r="H5" s="183"/>
+      <c r="I5" s="183"/>
     </row>
     <row r="6" spans="1:12" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="203" t="s">
+      <c r="A6" s="180" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="203"/>
-      <c r="C6" s="203"/>
-      <c r="D6" s="203"/>
-      <c r="E6" s="203"/>
-      <c r="F6" s="203"/>
-      <c r="G6" s="203"/>
-      <c r="H6" s="203"/>
-      <c r="I6" s="203"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="180"/>
+      <c r="D6" s="180"/>
+      <c r="E6" s="180"/>
+      <c r="F6" s="180"/>
+      <c r="G6" s="180"/>
+      <c r="H6" s="180"/>
+      <c r="I6" s="180"/>
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="195"/>
-      <c r="B7" s="195"/>
-      <c r="C7" s="195"/>
-      <c r="D7" s="195"/>
-      <c r="E7" s="195"/>
-      <c r="F7" s="195"/>
-      <c r="G7" s="195"/>
-      <c r="H7" s="195"/>
-      <c r="I7" s="195"/>
+      <c r="A7" s="185"/>
+      <c r="B7" s="185"/>
+      <c r="C7" s="185"/>
+      <c r="D7" s="185"/>
+      <c r="E7" s="185"/>
+      <c r="F7" s="185"/>
+      <c r="G7" s="185"/>
+      <c r="H7" s="185"/>
+      <c r="I7" s="185"/>
       <c r="L7" s="109"/>
     </row>
     <row r="8" spans="1:12" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="196" t="s">
+      <c r="A8" s="186" t="s">
         <v>779</v>
       </c>
-      <c r="B8" s="197"/>
-      <c r="C8" s="197"/>
-      <c r="D8" s="197"/>
-      <c r="E8" s="198"/>
+      <c r="B8" s="187"/>
+      <c r="C8" s="187"/>
+      <c r="D8" s="187"/>
+      <c r="E8" s="188"/>
       <c r="F8" s="110"/>
       <c r="G8" s="110"/>
       <c r="H8" s="110"/>
@@ -22486,12 +22486,12 @@
     </row>
     <row r="11" spans="1:12" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="116"/>
-      <c r="B11" s="199" t="s">
+      <c r="B11" s="189" t="s">
         <v>782</v>
       </c>
-      <c r="C11" s="199"/>
-      <c r="D11" s="199"/>
-      <c r="E11" s="200"/>
+      <c r="C11" s="189"/>
+      <c r="D11" s="189"/>
+      <c r="E11" s="190"/>
       <c r="F11" s="113">
         <f>'Condensed Financial Performance'!D18</f>
         <v>0</v>
@@ -22523,12 +22523,12 @@
     </row>
     <row r="12" spans="1:12" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="116"/>
-      <c r="B12" s="199" t="s">
+      <c r="B12" s="189" t="s">
         <v>783</v>
       </c>
-      <c r="C12" s="199"/>
-      <c r="D12" s="199"/>
-      <c r="E12" s="200"/>
+      <c r="C12" s="189"/>
+      <c r="D12" s="189"/>
+      <c r="E12" s="190"/>
       <c r="F12" s="113">
         <f>'Detailed Financial Performance'!F43</f>
         <v>0</v>
@@ -22560,12 +22560,12 @@
     </row>
     <row r="13" spans="1:12" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="116"/>
-      <c r="B13" s="199" t="s">
+      <c r="B13" s="189" t="s">
         <v>784</v>
       </c>
-      <c r="C13" s="199"/>
-      <c r="D13" s="199"/>
-      <c r="E13" s="200"/>
+      <c r="C13" s="189"/>
+      <c r="D13" s="189"/>
+      <c r="E13" s="190"/>
       <c r="F13" s="113">
         <f>'Condensed Financial Performance'!D14</f>
         <v>0</v>
@@ -22597,12 +22597,12 @@
     </row>
     <row r="14" spans="1:12" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="116"/>
-      <c r="B14" s="199" t="s">
+      <c r="B14" s="189" t="s">
         <v>785</v>
       </c>
-      <c r="C14" s="199"/>
-      <c r="D14" s="199"/>
-      <c r="E14" s="200"/>
+      <c r="C14" s="189"/>
+      <c r="D14" s="189"/>
+      <c r="E14" s="190"/>
       <c r="F14" s="113"/>
       <c r="G14" s="113"/>
       <c r="H14" s="113"/>
@@ -22613,12 +22613,12 @@
     </row>
     <row r="15" spans="1:12" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="116"/>
-      <c r="B15" s="199" t="s">
+      <c r="B15" s="189" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="199"/>
-      <c r="D15" s="199"/>
-      <c r="E15" s="200"/>
+      <c r="C15" s="189"/>
+      <c r="D15" s="189"/>
+      <c r="E15" s="190"/>
       <c r="F15" s="113"/>
       <c r="G15" s="113"/>
       <c r="H15" s="113"/>
@@ -22629,12 +22629,12 @@
     </row>
     <row r="16" spans="1:12" s="117" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="116"/>
-      <c r="B16" s="199" t="s">
+      <c r="B16" s="189" t="s">
         <v>786</v>
       </c>
-      <c r="C16" s="199"/>
-      <c r="D16" s="199"/>
-      <c r="E16" s="200"/>
+      <c r="C16" s="189"/>
+      <c r="D16" s="189"/>
+      <c r="E16" s="190"/>
       <c r="F16" s="113"/>
       <c r="G16" s="113"/>
       <c r="H16" s="113"/>
@@ -22645,12 +22645,12 @@
     </row>
     <row r="17" spans="1:13" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="116"/>
-      <c r="B17" s="201" t="s">
+      <c r="B17" s="191" t="s">
         <v>787</v>
       </c>
-      <c r="C17" s="201"/>
-      <c r="D17" s="201"/>
-      <c r="E17" s="202"/>
+      <c r="C17" s="191"/>
+      <c r="D17" s="191"/>
+      <c r="E17" s="192"/>
       <c r="F17" s="118">
         <f>SUM(F11:F16)</f>
         <v>0</v>
@@ -22698,12 +22698,12 @@
     </row>
     <row r="19" spans="1:13" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="116"/>
-      <c r="B19" s="181" t="s">
+      <c r="B19" s="184" t="s">
         <v>789</v>
       </c>
-      <c r="C19" s="181"/>
-      <c r="D19" s="181"/>
-      <c r="E19" s="182"/>
+      <c r="C19" s="184"/>
+      <c r="D19" s="184"/>
+      <c r="E19" s="193"/>
       <c r="F19"/>
       <c r="G19"/>
       <c r="H19"/>
@@ -22714,12 +22714,12 @@
     </row>
     <row r="20" spans="1:13" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="116"/>
-      <c r="B20" s="181" t="s">
+      <c r="B20" s="184" t="s">
         <v>790</v>
       </c>
-      <c r="C20" s="181"/>
-      <c r="D20" s="181"/>
-      <c r="E20" s="182"/>
+      <c r="C20" s="184"/>
+      <c r="D20" s="184"/>
+      <c r="E20" s="193"/>
       <c r="F20"/>
       <c r="G20"/>
       <c r="H20"/>
@@ -22730,12 +22730,12 @@
     </row>
     <row r="21" spans="1:13" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="116"/>
-      <c r="B21" s="181" t="s">
+      <c r="B21" s="184" t="s">
         <v>791</v>
       </c>
-      <c r="C21" s="181"/>
-      <c r="D21" s="181"/>
-      <c r="E21" s="181"/>
+      <c r="C21" s="184"/>
+      <c r="D21" s="184"/>
+      <c r="E21" s="184"/>
       <c r="F21" s="140">
         <f>'Condensed Financial Performance'!D20</f>
         <v>0</v>
@@ -22767,12 +22767,12 @@
     </row>
     <row r="22" spans="1:13" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="116"/>
-      <c r="B22" s="181" t="s">
+      <c r="B22" s="184" t="s">
         <v>792</v>
       </c>
-      <c r="C22" s="181"/>
-      <c r="D22" s="181"/>
-      <c r="E22" s="181"/>
+      <c r="C22" s="184"/>
+      <c r="D22" s="184"/>
+      <c r="E22" s="184"/>
       <c r="F22" s="140">
         <f>'Condensed Financial Performance'!D21</f>
         <v>0</v>
@@ -22804,12 +22804,12 @@
     </row>
     <row r="23" spans="1:13" s="117" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="116"/>
-      <c r="B23" s="181" t="s">
+      <c r="B23" s="184" t="s">
         <v>793</v>
       </c>
-      <c r="C23" s="181"/>
-      <c r="D23" s="181"/>
-      <c r="E23" s="181"/>
+      <c r="C23" s="184"/>
+      <c r="D23" s="184"/>
+      <c r="E23" s="184"/>
       <c r="F23" s="113">
         <f>'Condensed Financial Performance'!D22</f>
         <v>0</v>
@@ -22841,12 +22841,12 @@
     </row>
     <row r="24" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="116"/>
-      <c r="B24" s="183" t="s">
+      <c r="B24" s="194" t="s">
         <v>794</v>
       </c>
-      <c r="C24" s="183"/>
-      <c r="D24" s="183"/>
-      <c r="E24" s="183"/>
+      <c r="C24" s="194"/>
+      <c r="D24" s="194"/>
+      <c r="E24" s="194"/>
       <c r="F24" s="121">
         <f>SUM(F20:F23)</f>
         <v>0</v>
@@ -22948,12 +22948,12 @@
     </row>
     <row r="28" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="116"/>
-      <c r="B28" s="181" t="s">
+      <c r="B28" s="184" t="s">
         <v>797</v>
       </c>
-      <c r="C28" s="181"/>
-      <c r="D28" s="181"/>
-      <c r="E28" s="182"/>
+      <c r="C28" s="184"/>
+      <c r="D28" s="184"/>
+      <c r="E28" s="193"/>
       <c r="F28" s="113"/>
       <c r="G28" s="113"/>
       <c r="H28" s="113"/>
@@ -22964,12 +22964,12 @@
     </row>
     <row r="29" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="116"/>
-      <c r="B29" s="181" t="s">
+      <c r="B29" s="184" t="s">
         <v>798</v>
       </c>
-      <c r="C29" s="181"/>
-      <c r="D29" s="181"/>
-      <c r="E29" s="182"/>
+      <c r="C29" s="184"/>
+      <c r="D29" s="184"/>
+      <c r="E29" s="193"/>
       <c r="F29" s="113"/>
       <c r="G29" s="113"/>
       <c r="H29" s="113"/>
@@ -22980,12 +22980,12 @@
     </row>
     <row r="30" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="116"/>
-      <c r="B30" s="181" t="s">
+      <c r="B30" s="184" t="s">
         <v>799</v>
       </c>
-      <c r="C30" s="181"/>
-      <c r="D30" s="181"/>
-      <c r="E30" s="182"/>
+      <c r="C30" s="184"/>
+      <c r="D30" s="184"/>
+      <c r="E30" s="193"/>
       <c r="F30" s="113"/>
       <c r="G30" s="113"/>
       <c r="H30" s="113"/>
@@ -22996,12 +22996,12 @@
     </row>
     <row r="31" spans="1:13" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="116"/>
-      <c r="B31" s="181" t="s">
+      <c r="B31" s="184" t="s">
         <v>800</v>
       </c>
-      <c r="C31" s="181"/>
-      <c r="D31" s="181"/>
-      <c r="E31" s="182"/>
+      <c r="C31" s="184"/>
+      <c r="D31" s="184"/>
+      <c r="E31" s="193"/>
       <c r="F31" s="113"/>
       <c r="G31" s="113"/>
       <c r="H31" s="113"/>
@@ -23012,12 +23012,12 @@
     </row>
     <row r="32" spans="1:13" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="116"/>
-      <c r="B32" s="183" t="s">
+      <c r="B32" s="194" t="s">
         <v>787</v>
       </c>
-      <c r="C32" s="183"/>
-      <c r="D32" s="183"/>
-      <c r="E32" s="184"/>
+      <c r="C32" s="194"/>
+      <c r="D32" s="194"/>
+      <c r="E32" s="195"/>
       <c r="F32" s="118">
         <f>SUM(F28:F31)</f>
         <v>0</v>
@@ -23065,12 +23065,12 @@
     </row>
     <row r="34" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="116"/>
-      <c r="B34" s="181" t="s">
+      <c r="B34" s="184" t="s">
         <v>801</v>
       </c>
-      <c r="C34" s="181"/>
-      <c r="D34" s="181"/>
-      <c r="E34" s="182"/>
+      <c r="C34" s="184"/>
+      <c r="D34" s="184"/>
+      <c r="E34" s="193"/>
       <c r="F34" s="113">
         <f>'Financial Position'!D21</f>
         <v>0</v>
@@ -23102,12 +23102,12 @@
     </row>
     <row r="35" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="116"/>
-      <c r="B35" s="181" t="s">
+      <c r="B35" s="184" t="s">
         <v>802</v>
       </c>
-      <c r="C35" s="181"/>
-      <c r="D35" s="181"/>
-      <c r="E35" s="182"/>
+      <c r="C35" s="184"/>
+      <c r="D35" s="184"/>
+      <c r="E35" s="193"/>
       <c r="F35" s="113">
         <f>'Financial Position'!D22</f>
         <v>0</v>
@@ -23139,12 +23139,12 @@
     </row>
     <row r="36" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="116"/>
-      <c r="B36" s="181" t="s">
+      <c r="B36" s="184" t="s">
         <v>803</v>
       </c>
-      <c r="C36" s="181"/>
-      <c r="D36" s="181"/>
-      <c r="E36" s="182"/>
+      <c r="C36" s="184"/>
+      <c r="D36" s="184"/>
+      <c r="E36" s="193"/>
       <c r="F36" s="113"/>
       <c r="G36" s="113"/>
       <c r="H36" s="113"/>
@@ -23155,12 +23155,12 @@
     </row>
     <row r="37" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="116"/>
-      <c r="B37" s="181" t="s">
+      <c r="B37" s="184" t="s">
         <v>804</v>
       </c>
-      <c r="C37" s="181"/>
-      <c r="D37" s="181"/>
-      <c r="E37" s="182"/>
+      <c r="C37" s="184"/>
+      <c r="D37" s="184"/>
+      <c r="E37" s="193"/>
       <c r="F37" s="113"/>
       <c r="G37" s="113"/>
       <c r="H37" s="113"/>
@@ -23171,12 +23171,12 @@
     </row>
     <row r="38" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="116"/>
-      <c r="B38" s="181" t="s">
+      <c r="B38" s="184" t="s">
         <v>805</v>
       </c>
-      <c r="C38" s="181"/>
-      <c r="D38" s="181"/>
-      <c r="E38" s="182"/>
+      <c r="C38" s="184"/>
+      <c r="D38" s="184"/>
+      <c r="E38" s="193"/>
       <c r="F38" s="113"/>
       <c r="G38" s="113"/>
       <c r="H38" s="113"/>
@@ -23187,12 +23187,12 @@
     </row>
     <row r="39" spans="1:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="116"/>
-      <c r="B39" s="181" t="s">
+      <c r="B39" s="184" t="s">
         <v>806</v>
       </c>
-      <c r="C39" s="181"/>
-      <c r="D39" s="181"/>
-      <c r="E39" s="182"/>
+      <c r="C39" s="184"/>
+      <c r="D39" s="184"/>
+      <c r="E39" s="193"/>
       <c r="F39" s="113"/>
       <c r="G39" s="113"/>
       <c r="H39" s="113"/>
@@ -23203,12 +23203,12 @@
     </row>
     <row r="40" spans="1:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="116"/>
-      <c r="B40" s="183" t="s">
+      <c r="B40" s="194" t="s">
         <v>794</v>
       </c>
-      <c r="C40" s="183"/>
-      <c r="D40" s="183"/>
-      <c r="E40" s="184"/>
+      <c r="C40" s="194"/>
+      <c r="D40" s="194"/>
+      <c r="E40" s="195"/>
       <c r="F40" s="118">
         <f>SUM(F34:F39)</f>
         <v>0</v>
@@ -23307,12 +23307,12 @@
     </row>
     <row r="44" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="116"/>
-      <c r="B44" s="181" t="s">
+      <c r="B44" s="184" t="s">
         <v>809</v>
       </c>
-      <c r="C44" s="181"/>
-      <c r="D44" s="181"/>
-      <c r="E44" s="182"/>
+      <c r="C44" s="184"/>
+      <c r="D44" s="184"/>
+      <c r="E44" s="193"/>
       <c r="F44" s="113"/>
       <c r="G44" s="115"/>
       <c r="H44" s="113"/>
@@ -23322,12 +23322,12 @@
     </row>
     <row r="45" spans="1:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="116"/>
-      <c r="B45" s="181" t="s">
+      <c r="B45" s="184" t="s">
         <v>810</v>
       </c>
-      <c r="C45" s="181"/>
-      <c r="D45" s="181"/>
-      <c r="E45" s="182"/>
+      <c r="C45" s="184"/>
+      <c r="D45" s="184"/>
+      <c r="E45" s="193"/>
       <c r="F45" s="113"/>
       <c r="G45" s="115"/>
       <c r="H45" s="113"/>
@@ -23337,12 +23337,12 @@
     </row>
     <row r="46" spans="1:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="116"/>
-      <c r="B46" s="183" t="s">
+      <c r="B46" s="194" t="s">
         <v>787</v>
       </c>
-      <c r="C46" s="183"/>
-      <c r="D46" s="183"/>
-      <c r="E46" s="184"/>
+      <c r="C46" s="194"/>
+      <c r="D46" s="194"/>
+      <c r="E46" s="195"/>
       <c r="F46" s="118">
         <f>F44+F45</f>
         <v>0</v>
@@ -23389,12 +23389,12 @@
     </row>
     <row r="48" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="111"/>
-      <c r="B48" s="181" t="s">
+      <c r="B48" s="184" t="s">
         <v>811</v>
       </c>
-      <c r="C48" s="181"/>
-      <c r="D48" s="181"/>
-      <c r="E48" s="182"/>
+      <c r="C48" s="184"/>
+      <c r="D48" s="184"/>
+      <c r="E48" s="193"/>
       <c r="G48" s="115"/>
       <c r="H48" s="113"/>
       <c r="I48" s="113"/>
@@ -23403,12 +23403,12 @@
     </row>
     <row r="49" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="116"/>
-      <c r="B49" s="181" t="s">
+      <c r="B49" s="184" t="s">
         <v>812</v>
       </c>
-      <c r="C49" s="181"/>
-      <c r="D49" s="181"/>
-      <c r="E49" s="182"/>
+      <c r="C49" s="184"/>
+      <c r="D49" s="184"/>
+      <c r="E49" s="193"/>
       <c r="F49" s="113"/>
       <c r="G49" s="115"/>
       <c r="H49" s="113"/>
@@ -23418,12 +23418,12 @@
     </row>
     <row r="50" spans="1:15" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="116"/>
-      <c r="B50" s="181" t="s">
+      <c r="B50" s="184" t="s">
         <v>813</v>
       </c>
-      <c r="C50" s="181"/>
-      <c r="D50" s="181"/>
-      <c r="E50" s="182"/>
+      <c r="C50" s="184"/>
+      <c r="D50" s="184"/>
+      <c r="E50" s="193"/>
       <c r="F50" s="113"/>
       <c r="G50" s="115"/>
       <c r="H50" s="113"/>
@@ -23433,12 +23433,12 @@
     </row>
     <row r="51" spans="1:15" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="116"/>
-      <c r="B51" s="183" t="s">
+      <c r="B51" s="194" t="s">
         <v>794</v>
       </c>
-      <c r="C51" s="183"/>
-      <c r="D51" s="183"/>
-      <c r="E51" s="184"/>
+      <c r="C51" s="194"/>
+      <c r="D51" s="194"/>
+      <c r="E51" s="195"/>
       <c r="F51" s="118">
         <f>SUM(F48:F50)</f>
         <v>0</v>
@@ -23468,8 +23468,8 @@
         <v>0</v>
       </c>
       <c r="M51" s="129"/>
-      <c r="N51" s="192"/>
-      <c r="O51" s="193"/>
+      <c r="N51" s="196"/>
+      <c r="O51" s="197"/>
     </row>
     <row r="52" spans="1:15" s="127" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="122" t="s">
@@ -23507,17 +23507,17 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="N52" s="194"/>
-      <c r="O52" s="194"/>
+      <c r="N52" s="198"/>
+      <c r="O52" s="198"/>
     </row>
     <row r="53" spans="1:15" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="185" t="s">
+      <c r="A53" s="200" t="s">
         <v>815</v>
       </c>
-      <c r="B53" s="186"/>
-      <c r="C53" s="186"/>
-      <c r="D53" s="186"/>
-      <c r="E53" s="187"/>
+      <c r="B53" s="201"/>
+      <c r="C53" s="201"/>
+      <c r="D53" s="201"/>
+      <c r="E53" s="202"/>
       <c r="F53" s="130">
         <f>F25+F41</f>
         <v>0</v>
@@ -23549,13 +23549,13 @@
       <c r="M53" s="109"/>
     </row>
     <row r="54" spans="1:15" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="185" t="s">
+      <c r="A54" s="200" t="s">
         <v>816</v>
       </c>
-      <c r="B54" s="186"/>
-      <c r="C54" s="186"/>
-      <c r="D54" s="186"/>
-      <c r="E54" s="187"/>
+      <c r="B54" s="201"/>
+      <c r="C54" s="201"/>
+      <c r="D54" s="201"/>
+      <c r="E54" s="202"/>
       <c r="F54" s="131"/>
       <c r="G54" s="131"/>
       <c r="H54" s="131"/>
@@ -23566,13 +23566,13 @@
       <c r="M54" s="109"/>
     </row>
     <row r="55" spans="1:15" s="133" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="188" t="s">
+      <c r="A55" s="203" t="s">
         <v>817</v>
       </c>
-      <c r="B55" s="189"/>
-      <c r="C55" s="189"/>
-      <c r="D55" s="189"/>
-      <c r="E55" s="190"/>
+      <c r="B55" s="204"/>
+      <c r="C55" s="204"/>
+      <c r="D55" s="204"/>
+      <c r="E55" s="205"/>
       <c r="F55" s="132">
         <f>F53+F54</f>
         <v>0</v>
@@ -23629,7 +23629,7 @@
       <c r="B59" s="161"/>
       <c r="C59" s="161"/>
       <c r="D59" s="161"/>
-      <c r="E59" s="191" t="s">
+      <c r="E59" s="206" t="s">
         <v>819</v>
       </c>
       <c r="F59" s="161"/>
@@ -23641,15 +23641,15 @@
       <c r="N59" s="109"/>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A60" s="180"/>
-      <c r="B60" s="180"/>
-      <c r="C60" s="180"/>
-      <c r="D60" s="180"/>
-      <c r="E60" s="180" t="s">
+      <c r="A60" s="199"/>
+      <c r="B60" s="199"/>
+      <c r="C60" s="199"/>
+      <c r="D60" s="199"/>
+      <c r="E60" s="199" t="s">
         <v>29</v>
       </c>
-      <c r="F60" s="180"/>
-      <c r="G60" s="180"/>
+      <c r="F60" s="199"/>
+      <c r="G60" s="199"/>
       <c r="H60" s="3"/>
       <c r="I60" s="3"/>
       <c r="L60" s="109"/>
@@ -23671,12 +23671,37 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="E60:G60"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B36:E36"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="A8:E8"/>
@@ -23689,37 +23714,12 @@
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="E60:G60"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A5:I5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="67" orientation="portrait" r:id="rId1"/>

</xml_diff>